<commit_message>
fix: mejoras en los alerts de sweet alert 2
</commit_message>
<xml_diff>
--- a/frontend/public/excels/horarios.xlsx
+++ b/frontend/public/excels/horarios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88AD8389-8554-4498-A62D-C58931E70D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACAEA7D-EA86-4CE2-996D-D38C835E4736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Semestre 2" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2529" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2692" uniqueCount="337">
   <si>
     <t>NRC</t>
   </si>
@@ -962,6 +962,81 @@
   </si>
   <si>
     <t>TENDENCIAS TECNOL. EN LAS TIC</t>
+  </si>
+  <si>
+    <t>24826</t>
+  </si>
+  <si>
+    <t>I001</t>
+  </si>
+  <si>
+    <t>PRACTICA PROFESIONAL</t>
+  </si>
+  <si>
+    <t>24150</t>
+  </si>
+  <si>
+    <t>24151</t>
+  </si>
+  <si>
+    <t>PABLO</t>
+  </si>
+  <si>
+    <t>COELHO/CARO</t>
+  </si>
+  <si>
+    <t>24152</t>
+  </si>
+  <si>
+    <t>SEBASTIAN</t>
+  </si>
+  <si>
+    <t>PONS/VARGAS</t>
+  </si>
+  <si>
+    <t>24153</t>
+  </si>
+  <si>
+    <t>14383</t>
+  </si>
+  <si>
+    <t>0018</t>
+  </si>
+  <si>
+    <t>ECUACIONES DIFERENCIALES</t>
+  </si>
+  <si>
+    <t>14395</t>
+  </si>
+  <si>
+    <t>T1E</t>
+  </si>
+  <si>
+    <t>21693</t>
+  </si>
+  <si>
+    <t>J003</t>
+  </si>
+  <si>
+    <t>SEGURIDAD INFORMATICA</t>
+  </si>
+  <si>
+    <t>SILVIA</t>
+  </si>
+  <si>
+    <t>REYES/QUEZADA/</t>
+  </si>
+  <si>
+    <t>21694</t>
+  </si>
+  <si>
+    <t>1434</t>
+  </si>
+  <si>
+    <t>GESTION ESTRATEGICA</t>
+  </si>
+  <si>
+    <t>13914</t>
   </si>
 </sst>
 </file>
@@ -1391,13 +1466,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B04450B-4D3A-444A-8C70-833821F0E18C}">
   <dimension ref="A1:S33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -2972,13 +3047,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742B1EB3-54E8-42B1-96A5-AD861CB086AD}">
-  <dimension ref="A1:S21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:S31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -3511,102 +3586,98 @@
       <c r="S11" s="2"/>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="6">
-        <v>24555</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="6">
-        <v>6</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="J12" s="6">
-        <v>1440</v>
-      </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6" t="s">
+      <c r="A12" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R12" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S12" s="6"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="13" spans="1:19">
-      <c r="A13" s="6">
-        <v>24555</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="6">
-        <v>6</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="J13" s="6">
-        <v>1610</v>
-      </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R13" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S13" s="6"/>
+      <c r="A13" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="S13" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="14" spans="1:19">
       <c r="A14" s="6">
-        <v>24556</v>
+        <v>24555</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>287</v>
@@ -3618,7 +3689,7 @@
         <v>6</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>49</v>
@@ -3629,7 +3700,7 @@
       <c r="H14" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="7" t="s">
         <v>34</v>
       </c>
       <c r="J14" s="6">
@@ -3642,7 +3713,7 @@
         <v>29</v>
       </c>
       <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
+      <c r="P14" s="7"/>
       <c r="Q14" s="6" t="s">
         <v>102</v>
       </c>
@@ -3653,7 +3724,7 @@
     </row>
     <row r="15" spans="1:19">
       <c r="A15" s="6">
-        <v>24556</v>
+        <v>24555</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>287</v>
@@ -3665,7 +3736,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>49</v>
@@ -3676,7 +3747,7 @@
       <c r="H15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="7" t="s">
         <v>34</v>
       </c>
       <c r="J15" s="6">
@@ -3689,7 +3760,7 @@
         <v>29</v>
       </c>
       <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
+      <c r="P15" s="7"/>
       <c r="Q15" s="6" t="s">
         <v>102</v>
       </c>
@@ -3700,7 +3771,7 @@
     </row>
     <row r="16" spans="1:19">
       <c r="A16" s="6">
-        <v>24557</v>
+        <v>24556</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>287</v>
@@ -3712,7 +3783,7 @@
         <v>6</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>49</v>
@@ -3721,22 +3792,22 @@
         <v>208</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>24</v>
+        <v>81</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="J16" s="6">
-        <v>1311</v>
+        <v>1440</v>
       </c>
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
       <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="P16" s="6"/>
+      <c r="N16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="O16" s="6"/>
+      <c r="P16" s="7"/>
       <c r="Q16" s="6" t="s">
         <v>102</v>
       </c>
@@ -3747,7 +3818,7 @@
     </row>
     <row r="17" spans="1:19">
       <c r="A17" s="6">
-        <v>24557</v>
+        <v>24556</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>287</v>
@@ -3759,7 +3830,7 @@
         <v>6</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>49</v>
@@ -3768,22 +3839,22 @@
         <v>208</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>24</v>
+        <v>81</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="J17" s="6">
-        <v>1440</v>
+        <v>1610</v>
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="P17" s="6"/>
+      <c r="N17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="O17" s="6"/>
+      <c r="P17" s="7"/>
       <c r="Q17" s="6" t="s">
         <v>102</v>
       </c>
@@ -3794,7 +3865,7 @@
     </row>
     <row r="18" spans="1:19">
       <c r="A18" s="6">
-        <v>24559</v>
+        <v>24557</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>287</v>
@@ -3806,7 +3877,7 @@
         <v>6</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>49</v>
@@ -3817,7 +3888,7 @@
       <c r="H18" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" s="7" t="s">
         <v>24</v>
       </c>
       <c r="J18" s="6">
@@ -3830,7 +3901,7 @@
       <c r="O18" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="P18" s="6"/>
+      <c r="P18" s="7"/>
       <c r="Q18" s="6" t="s">
         <v>102</v>
       </c>
@@ -3841,7 +3912,7 @@
     </row>
     <row r="19" spans="1:19">
       <c r="A19" s="6">
-        <v>24559</v>
+        <v>24557</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>287</v>
@@ -3853,7 +3924,7 @@
         <v>6</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>49</v>
@@ -3864,7 +3935,7 @@
       <c r="H19" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="7" t="s">
         <v>24</v>
       </c>
       <c r="J19" s="6">
@@ -3877,7 +3948,7 @@
       <c r="O19" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="P19" s="6"/>
+      <c r="P19" s="7"/>
       <c r="Q19" s="6" t="s">
         <v>102</v>
       </c>
@@ -3887,114 +3958,584 @@
       <c r="S19" s="6"/>
     </row>
     <row r="20" spans="1:19">
-      <c r="A20" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="A20" s="6">
+        <v>24559</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="6">
+        <v>6</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J20" s="6">
+        <v>1311</v>
+      </c>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S20" s="6"/>
+    </row>
+    <row r="21" spans="1:19">
+      <c r="A21" s="6">
+        <v>24559</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="6">
+        <v>6</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J21" s="6">
+        <v>1440</v>
+      </c>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S21" s="6"/>
+    </row>
+    <row r="22" spans="1:19">
+      <c r="A22" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S22" s="6"/>
+    </row>
+    <row r="23" spans="1:19">
+      <c r="A23" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R23" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S23" s="6"/>
+    </row>
+    <row r="24" spans="1:19">
+      <c r="A24" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="R20" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="S20" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19">
-      <c r="A21" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="G24" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="S24" s="1"/>
+    </row>
+    <row r="25" spans="1:19">
+      <c r="A25" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1" t="s">
+      <c r="G25" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="S25" s="1"/>
+    </row>
+    <row r="26" spans="1:19">
+      <c r="A26" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="R21" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>96</v>
-      </c>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="S26" s="1"/>
+    </row>
+    <row r="27" spans="1:19">
+      <c r="A27" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="S27" s="1"/>
+    </row>
+    <row r="28" spans="1:19">
+      <c r="A28" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="S28" s="1"/>
+    </row>
+    <row r="29" spans="1:19">
+      <c r="A29" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="S29" s="1"/>
+    </row>
+    <row r="30" spans="1:19">
+      <c r="A30" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="7"/>
+      <c r="Q30" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R30" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S30" s="6"/>
+    </row>
+    <row r="31" spans="1:19">
+      <c r="A31" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="7"/>
+      <c r="Q31" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R31" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S31" s="6"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S11">
-    <sortCondition ref="A2:A11"/>
-    <sortCondition ref="J2:J11"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31639A8-B77F-40D3-A3E2-D8298BF83C8B}">
-  <dimension ref="A1:S33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:S30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="5.85546875" customWidth="1"/>
-    <col min="7" max="7" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" customWidth="1"/>
+    <col min="7" max="7" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -4156,7 +4697,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="1" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>287</v>
@@ -4165,7 +4706,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>63</v>
@@ -4174,36 +4715,36 @@
         <v>43</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>33</v>
+        <v>92</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1" t="s">
-        <v>41</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1" t="s">
-        <v>37</v>
+        <v>175</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>38</v>
+        <v>176</v>
       </c>
       <c r="S4" s="1"/>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="1" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>287</v>
@@ -4212,7 +4753,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>63</v>
@@ -4221,36 +4762,38 @@
         <v>43</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>33</v>
+        <v>92</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="N5" s="1"/>
-      <c r="O5" s="1" t="s">
-        <v>56</v>
-      </c>
+      <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1" t="s">
-        <v>37</v>
+        <v>175</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="S5" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="1" t="s">
-        <v>125</v>
+        <v>177</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>287</v>
@@ -4259,45 +4802,45 @@
         <v>18</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" s="1" t="s">
-        <v>36</v>
-      </c>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
+      <c r="O6" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1" t="s">
-        <v>37</v>
+        <v>163</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>38</v>
+        <v>164</v>
       </c>
       <c r="S6" s="1"/>
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="1" t="s">
-        <v>126</v>
+        <v>177</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>287</v>
@@ -4306,45 +4849,45 @@
         <v>18</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>122</v>
+        <v>42</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="K7" s="1"/>
-      <c r="L7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1" t="s">
-        <v>85</v>
+        <v>163</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="1" t="s">
-        <v>126</v>
+        <v>177</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>287</v>
@@ -4353,45 +4896,45 @@
         <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>122</v>
+        <v>42</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
-      <c r="O8" s="1" t="s">
-        <v>56</v>
-      </c>
+      <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1" t="s">
-        <v>85</v>
+        <v>163</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="S8" s="1"/>
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="1" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>287</v>
@@ -4400,45 +4943,47 @@
         <v>18</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="1" t="s">
-        <v>36</v>
-      </c>
+      <c r="M9" s="1"/>
       <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
+      <c r="O9" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="S9" s="1"/>
+        <v>60</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="10" spans="1:19">
       <c r="A10" s="1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>287</v>
@@ -4447,25 +4992,25 @@
         <v>18</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>89</v>
+        <v>178</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>90</v>
+        <v>179</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>26</v>
@@ -4476,16 +5021,16 @@
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1" t="s">
-        <v>175</v>
+        <v>59</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>176</v>
+        <v>60</v>
       </c>
       <c r="S10" s="1"/>
     </row>
     <row r="11" spans="1:19">
       <c r="A11" s="1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>287</v>
@@ -4494,25 +5039,25 @@
         <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>89</v>
+        <v>178</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>90</v>
+        <v>179</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -4523,654 +5068,644 @@
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1" t="s">
-        <v>175</v>
+        <v>59</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>176</v>
+        <v>60</v>
       </c>
       <c r="S11" s="1" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="A12" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
+      <c r="A13" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
+      <c r="A14" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19">
+      <c r="A15" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19">
+      <c r="A16" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="S16" s="2"/>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="S17" s="2"/>
+    </row>
+    <row r="18" spans="1:19">
+      <c r="A18" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19">
+      <c r="A19" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19">
+      <c r="A20" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="S20" s="2"/>
+    </row>
+    <row r="21" spans="1:19">
+      <c r="A21" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="S21" s="2"/>
+    </row>
+    <row r="22" spans="1:19">
+      <c r="A22" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H12" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="R12" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S12" s="1"/>
-    </row>
-    <row r="13" spans="1:19">
-      <c r="A13" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S13" s="1"/>
-    </row>
-    <row r="14" spans="1:19">
-      <c r="A14" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S14" s="1"/>
-    </row>
-    <row r="15" spans="1:19">
-      <c r="A15" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19">
-      <c r="A16" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="S16" s="1"/>
-    </row>
-    <row r="17" spans="1:19">
-      <c r="A17" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="R17" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19">
-      <c r="A18" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q18" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R18" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S18" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19">
-      <c r="A19" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q19" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R19" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S19" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19">
-      <c r="A20" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q20" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R20" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S20" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19">
-      <c r="A21" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q21" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="R21" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="S21" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19">
-      <c r="A22" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2" t="s">
+      <c r="I22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="S22" s="2"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="S22" s="1"/>
     </row>
     <row r="23" spans="1:19">
       <c r="A23" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B23" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>287</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+        <v>218</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="J23" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
+      <c r="L23" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="M23" s="2"/>
-      <c r="N23" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>186</v>
+        <v>84</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>187</v>
+        <v>221</v>
       </c>
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:19">
       <c r="A24" s="2" t="s">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>287</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+        <v>218</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="J24" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
+      <c r="L24" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="M24" s="2"/>
-      <c r="N24" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
       <c r="Q24" s="2" t="s">
-        <v>189</v>
+        <v>84</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="S24" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="S24" s="2"/>
     </row>
     <row r="25" spans="1:19">
       <c r="A25" s="2" t="s">
-        <v>188</v>
+        <v>222</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>287</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+        <v>218</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="J25" s="2" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -5181,384 +5716,251 @@
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
       <c r="Q25" s="2" t="s">
-        <v>189</v>
+        <v>84</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="S25" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="S25" s="2"/>
     </row>
     <row r="26" spans="1:19">
       <c r="A26" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B26" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>287</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
+        <v>218</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="J26" s="2" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="M26" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
       <c r="Q26" s="2" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>191</v>
+        <v>221</v>
       </c>
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="1:19">
       <c r="A27" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B27" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>287</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K27" s="2"/>
+      <c r="K27" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
-      <c r="N27" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
       <c r="Q27" s="2" t="s">
-        <v>101</v>
+        <v>244</v>
       </c>
       <c r="R27" s="2" t="s">
-        <v>191</v>
+        <v>245</v>
       </c>
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="1:19">
       <c r="A28" s="1" t="s">
-        <v>217</v>
+        <v>323</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>145</v>
+        <v>324</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>43</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>218</v>
+        <v>325</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="K28" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
-      <c r="N28" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="N28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="1" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="S28" s="1"/>
+        <v>164</v>
+      </c>
+      <c r="S28" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="29" spans="1:19">
-      <c r="A29" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="A29" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="S29" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="S29" s="2"/>
     </row>
     <row r="30" spans="1:19">
       <c r="A30" s="2" t="s">
-        <v>220</v>
+        <v>326</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>287</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>145</v>
+        <v>324</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>20</v>
+        <v>327</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>218</v>
+        <v>325</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="K30" s="2"/>
-      <c r="L30" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="M30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="2" t="s">
-        <v>84</v>
+        <v>163</v>
       </c>
       <c r="R30" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="S30" s="2"/>
-    </row>
-    <row r="31" spans="1:19">
-      <c r="A31" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="S30" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="S31" s="2"/>
-    </row>
-    <row r="32" spans="1:19">
-      <c r="A32" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="R32" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="S32" s="2"/>
-    </row>
-    <row r="33" spans="1:19">
-      <c r="A33" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="S33" s="2"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S3">
-    <sortCondition ref="A2:A3"/>
-    <sortCondition ref="J2:J3"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5566,13 +5968,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36BD2444-5417-4C3B-ACAC-17D64029070C}">
   <dimension ref="A1:S33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="7" max="7" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="18" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -7054,15 +7456,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ABF100-BEC0-4DD6-AD50-C4B8A3F777CB}">
   <dimension ref="A1:S47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.5546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -9177,16 +9578,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BE4429E-CA1B-4529-94AE-CE97ED6F115A}">
-  <dimension ref="A1:S28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:S29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="32.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -10333,8 +10733,8 @@
       <c r="I25" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>74</v>
+      <c r="J25" s="1">
+        <v>1311</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -10427,8 +10827,8 @@
       <c r="I27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>74</v>
+      <c r="J27" s="1">
+        <v>1311</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
@@ -10492,6 +10892,45 @@
         <v>253</v>
       </c>
       <c r="S28" s="6"/>
+    </row>
+    <row r="29" spans="1:19">
+      <c r="A29" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="R29" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="S29" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10500,16 +10939,16 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939E82A5-8A64-4B2B-8701-1D6FF57E175E}">
-  <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:S17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -11052,6 +11491,235 @@
       </c>
       <c r="S12" s="1"/>
     </row>
+    <row r="13" spans="1:19">
+      <c r="A13" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="S13" s="1"/>
+    </row>
+    <row r="14" spans="1:19">
+      <c r="A14" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="S14" s="6"/>
+    </row>
+    <row r="15" spans="1:19">
+      <c r="A15" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="S15" s="6"/>
+    </row>
+    <row r="16" spans="1:19">
+      <c r="A16" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="S16" s="1"/>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="S17" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>